<commit_message>
updated and corrected the longitude and latitude values for the following communes in Wilaya of Laghouat
</commit_message>
<xml_diff>
--- a/excel/algeria_cities.xlsx
+++ b/excel/algeria_cities.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\02 Donnees geographiques\algeria cities\Github\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EE2F4593-A359-492C-8F9D-DB9A636A3E37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{750BE355-39D4-4B33-ACB3-07B34DA945DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DBF91C95-A10C-4DD3-8A9B-F5B95CC12962}"/>
+    <workbookView xWindow="690" yWindow="3405" windowWidth="16410" windowHeight="11295" xr2:uid="{DBF91C95-A10C-4DD3-8A9B-F5B95CC12962}"/>
   </bookViews>
   <sheets>
     <sheet name="algeria_cities" sheetId="1" r:id="rId1"/>
@@ -12174,10 +12174,10 @@
         <v>311</v>
       </c>
       <c r="J55">
-        <v>34.184317999999998</v>
+        <v>34.156872</v>
       </c>
       <c r="K55">
-        <v>1.54179</v>
+        <v>1.542386</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.25">
@@ -12524,10 +12524,10 @@
         <v>545</v>
       </c>
       <c r="J65">
-        <v>33.722499999999997</v>
+        <v>33.645394000000003</v>
       </c>
       <c r="K65">
-        <v>3.19306</v>
+        <v>2.4447130000000001</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.25">
@@ -12594,10 +12594,10 @@
         <v>303</v>
       </c>
       <c r="J67">
-        <v>33.75</v>
+        <v>33.751463000000001</v>
       </c>
       <c r="K67">
-        <v>3.4472200000000002</v>
+        <v>3.002939</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.25">
@@ -61139,10 +61139,10 @@
         <v>314</v>
       </c>
       <c r="J1454">
-        <v>33.933332999999998</v>
+        <v>33.930145000000003</v>
       </c>
       <c r="K1454">
-        <v>2.9462999999999999</v>
+        <v>2.1407029999999998</v>
       </c>
     </row>
     <row r="1455" spans="1:11" x14ac:dyDescent="0.25">

</xml_diff>